<commit_message>
sửa import + lịch dạy giảng viên
</commit_message>
<xml_diff>
--- a/backend/sample_data/schedule_gv001_test.xlsx
+++ b/backend/sample_data/schedule_gv001_test.xlsx
@@ -1,41 +1,170 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Tai_lieu_hoc_tap\code\SIC-project\backend\sample_data\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BE65434-68F8-4041-A8FE-CF5432F5951C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="16220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
     <sheet name="ThoiKhoaBieu" sheetId="1" r:id="rId1"/>
   </sheets>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="46">
+  <si>
+    <t>Mã Môn</t>
+  </si>
+  <si>
+    <t>Tên Môn</t>
+  </si>
+  <si>
+    <t>Số Tín Chỉ</t>
+  </si>
+  <si>
+    <t>Mã Lớp HP</t>
+  </si>
+  <si>
+    <t>Học Kỳ</t>
+  </si>
+  <si>
+    <t>Năm Học</t>
+  </si>
+  <si>
+    <t>Mã GV</t>
+  </si>
+  <si>
+    <t>Phòng Học</t>
+  </si>
+  <si>
+    <t>Giờ Bắt Đầu</t>
+  </si>
+  <si>
+    <t>Giờ Kết Thúc</t>
+  </si>
+  <si>
+    <t>Ngày Bắt Đầu</t>
+  </si>
+  <si>
+    <t>Tổng Số Buổi</t>
+  </si>
+  <si>
+    <t>Danh Sách MSSV</t>
+  </si>
+  <si>
+    <t>INT3306</t>
+  </si>
+  <si>
+    <t>Phát Triển Ứng Dụng Web</t>
+  </si>
+  <si>
+    <t>INT3306_01</t>
+  </si>
+  <si>
+    <t>HK1</t>
+  </si>
+  <si>
+    <t>2026-2027</t>
+  </si>
+  <si>
+    <t>GV001</t>
+  </si>
+  <si>
+    <t>A2-301</t>
+  </si>
+  <si>
+    <t>07:00</t>
+  </si>
+  <si>
+    <t>09:15</t>
+  </si>
+  <si>
+    <t>2026-08-24</t>
+  </si>
+  <si>
+    <t>21020001, 21020002, 21020003, 21020004</t>
+  </si>
+  <si>
+    <t>INT3308</t>
+  </si>
+  <si>
+    <t>Thị Giác Máy Tính &amp; AI</t>
+  </si>
+  <si>
+    <t>INT3308_01</t>
+  </si>
+  <si>
+    <t>B1-102</t>
+  </si>
+  <si>
+    <t>2026-08-25</t>
+  </si>
+  <si>
+    <t>21020001, 21020002, 21020005, 21020088</t>
+  </si>
+  <si>
+    <t>INT3310</t>
+  </si>
+  <si>
+    <t>Lập Trình Python Chuyên Sâu</t>
+  </si>
+  <si>
+    <t>INT3310_01</t>
+  </si>
+  <si>
+    <t>09:30</t>
+  </si>
+  <si>
+    <t>11:45</t>
+  </si>
+  <si>
+    <t>21020003, 21020004, 21020099, 21020100</t>
+  </si>
+  <si>
+    <t>INT3315</t>
+  </si>
+  <si>
+    <t>Trí Tuệ Nhân Tạo Nâng Cao</t>
+  </si>
+  <si>
+    <t>INT3315_01</t>
+  </si>
+  <si>
+    <t>2026-08-27</t>
+  </si>
+  <si>
+    <t>21020001, 21020005, 21020088, 21020099</t>
+  </si>
+  <si>
+    <t>INT3320</t>
+  </si>
+  <si>
+    <t>Xử Lý Ngôn Ngữ Tự Nhiên</t>
+  </si>
+  <si>
+    <t>INT3320_01</t>
+  </si>
+  <si>
+    <t>2026-08-28</t>
+  </si>
+  <si>
+    <t>21020002, 21020004, 21020088, 21020100</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-  </numFmts>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -64,14 +193,23 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+  <cellXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -396,258 +534,271 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:M6"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="25.08203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.58203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.58203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.1640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.83203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.4140625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="36" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Mã Môn</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Tên Môn</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Số Tín Chỉ</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Mã Lớp HP</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Học Kỳ</v>
-      </c>
-      <c r="F1" t="str">
-        <v>Năm Học</v>
-      </c>
-      <c r="G1" t="str">
-        <v>Mã GV</v>
-      </c>
-      <c r="H1" t="str">
-        <v>Phòng Học</v>
-      </c>
-      <c r="I1" t="str">
-        <v>Giờ Bắt Đầu</v>
-      </c>
-      <c r="J1" t="str">
-        <v>Giờ Kết Thúc</v>
-      </c>
-      <c r="K1" t="str">
-        <v>Ngày Bắt Đầu</v>
-      </c>
-      <c r="L1" t="str">
-        <v>Tổng Số Buổi</v>
-      </c>
-      <c r="M1" t="str">
-        <v>Danh Sách MSSV</v>
+    <row r="1" spans="1:13" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" t="s">
+        <v>12</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>INT3306</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Phát Triển Ứng Dụng Web</v>
+    <row r="2" spans="1:13" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2" t="s">
+        <v>14</v>
       </c>
       <c r="C2">
         <v>3</v>
       </c>
-      <c r="D2" t="str">
-        <v>INT3306_01</v>
-      </c>
-      <c r="E2" t="str">
-        <v>HK1</v>
-      </c>
-      <c r="F2" t="str">
-        <v>2026-2027</v>
-      </c>
-      <c r="G2" t="str">
-        <v>GV001</v>
-      </c>
-      <c r="H2" t="str">
-        <v>A2-301</v>
-      </c>
-      <c r="I2" t="str">
-        <v>07:00</v>
-      </c>
-      <c r="J2" t="str">
-        <v>09:15</v>
-      </c>
-      <c r="K2" t="str">
-        <v>2026-08-24</v>
+      <c r="D2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G2" t="s">
+        <v>18</v>
+      </c>
+      <c r="H2" t="s">
+        <v>19</v>
+      </c>
+      <c r="I2" t="s">
+        <v>20</v>
+      </c>
+      <c r="J2" t="s">
+        <v>21</v>
+      </c>
+      <c r="K2" t="s">
+        <v>22</v>
       </c>
       <c r="L2">
         <v>15</v>
       </c>
-      <c r="M2" t="str">
-        <v>21020001, 21020002, 21020003, 21020004</v>
+      <c r="M2" t="s">
+        <v>23</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>INT3308</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Thị Giác Máy Tính &amp; AI</v>
+    <row r="3" spans="1:13" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B3" t="s">
+        <v>25</v>
       </c>
       <c r="C3">
         <v>3</v>
       </c>
-      <c r="D3" t="str">
-        <v>INT3308_01</v>
-      </c>
-      <c r="E3" t="str">
-        <v>HK1</v>
-      </c>
-      <c r="F3" t="str">
-        <v>2026-2027</v>
-      </c>
-      <c r="G3" t="str">
-        <v>GV001</v>
-      </c>
-      <c r="H3" t="str">
-        <v>B1-102</v>
-      </c>
-      <c r="I3" t="str">
-        <v>07:00</v>
-      </c>
-      <c r="J3" t="str">
-        <v>09:15</v>
-      </c>
-      <c r="K3" t="str">
-        <v>2026-08-25</v>
+      <c r="D3" t="s">
+        <v>26</v>
+      </c>
+      <c r="E3" t="s">
+        <v>16</v>
+      </c>
+      <c r="F3" t="s">
+        <v>17</v>
+      </c>
+      <c r="G3" t="s">
+        <v>18</v>
+      </c>
+      <c r="H3" t="s">
+        <v>27</v>
+      </c>
+      <c r="I3" t="s">
+        <v>20</v>
+      </c>
+      <c r="J3" t="s">
+        <v>21</v>
+      </c>
+      <c r="K3" t="s">
+        <v>28</v>
       </c>
       <c r="L3">
         <v>15</v>
       </c>
-      <c r="M3" t="str">
-        <v>21020001, 21020002, 21020005, 21020088</v>
+      <c r="M3" t="s">
+        <v>29</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>INT3310</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Lập Trình Python Chuyên Sâu</v>
+    <row r="4" spans="1:13" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B4" t="s">
+        <v>31</v>
       </c>
       <c r="C4">
         <v>3</v>
       </c>
-      <c r="D4" t="str">
-        <v>INT3310_01</v>
-      </c>
-      <c r="E4" t="str">
-        <v>HK1</v>
-      </c>
-      <c r="F4" t="str">
-        <v>2026-2027</v>
-      </c>
-      <c r="G4" t="str">
-        <v>GV001</v>
-      </c>
-      <c r="H4" t="str">
-        <v>A2-301</v>
-      </c>
-      <c r="I4" t="str">
-        <v>09:30</v>
-      </c>
-      <c r="J4" t="str">
-        <v>11:45</v>
-      </c>
-      <c r="K4" t="str">
-        <v>2026-08-25</v>
+      <c r="D4" t="s">
+        <v>32</v>
+      </c>
+      <c r="E4" t="s">
+        <v>16</v>
+      </c>
+      <c r="F4" t="s">
+        <v>17</v>
+      </c>
+      <c r="G4" t="s">
+        <v>18</v>
+      </c>
+      <c r="H4" t="s">
+        <v>19</v>
+      </c>
+      <c r="I4" t="s">
+        <v>33</v>
+      </c>
+      <c r="J4" t="s">
+        <v>34</v>
+      </c>
+      <c r="K4" t="s">
+        <v>28</v>
       </c>
       <c r="L4">
         <v>15</v>
       </c>
-      <c r="M4" t="str">
-        <v>21020003, 21020004, 21020099, 21020100</v>
+      <c r="M4" t="s">
+        <v>35</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>INT3315</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Trí Tuệ Nhân Tạo Nâng Cao</v>
+    <row r="5" spans="1:13" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>36</v>
+      </c>
+      <c r="B5" t="s">
+        <v>37</v>
       </c>
       <c r="C5">
         <v>3</v>
       </c>
-      <c r="D5" t="str">
-        <v>INT3315_01</v>
-      </c>
-      <c r="E5" t="str">
-        <v>HK1</v>
-      </c>
-      <c r="F5" t="str">
-        <v>2026-2027</v>
-      </c>
-      <c r="G5" t="str">
-        <v>GV001</v>
-      </c>
-      <c r="H5" t="str">
-        <v>B1-102</v>
-      </c>
-      <c r="I5" t="str">
-        <v>13:00</v>
-      </c>
-      <c r="J5" t="str">
-        <v>15:15</v>
-      </c>
-      <c r="K5" t="str">
-        <v>2026-08-27</v>
+      <c r="D5" t="s">
+        <v>38</v>
+      </c>
+      <c r="E5" t="s">
+        <v>16</v>
+      </c>
+      <c r="F5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G5" t="s">
+        <v>18</v>
+      </c>
+      <c r="H5" t="s">
+        <v>27</v>
+      </c>
+      <c r="I5" s="1">
+        <v>0.875</v>
+      </c>
+      <c r="J5" s="1">
+        <v>0.96875</v>
+      </c>
+      <c r="K5" t="s">
+        <v>39</v>
       </c>
       <c r="L5">
         <v>15</v>
       </c>
-      <c r="M5" t="str">
-        <v>21020001, 21020005, 21020088, 21020099</v>
+      <c r="M5" t="s">
+        <v>40</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>INT3320</v>
-      </c>
-      <c r="B6" t="str">
-        <v>Xử Lý Ngôn Ngữ Tự Nhiên</v>
+    <row r="6" spans="1:13" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>41</v>
+      </c>
+      <c r="B6" t="s">
+        <v>42</v>
       </c>
       <c r="C6">
         <v>3</v>
       </c>
-      <c r="D6" t="str">
-        <v>INT3320_01</v>
-      </c>
-      <c r="E6" t="str">
-        <v>HK1</v>
-      </c>
-      <c r="F6" t="str">
-        <v>2026-2027</v>
-      </c>
-      <c r="G6" t="str">
-        <v>GV001</v>
-      </c>
-      <c r="H6" t="str">
-        <v>A2-301</v>
-      </c>
-      <c r="I6" t="str">
-        <v>07:00</v>
-      </c>
-      <c r="J6" t="str">
-        <v>09:15</v>
-      </c>
-      <c r="K6" t="str">
-        <v>2026-08-28</v>
+      <c r="D6" t="s">
+        <v>43</v>
+      </c>
+      <c r="E6" t="s">
+        <v>16</v>
+      </c>
+      <c r="F6" t="s">
+        <v>17</v>
+      </c>
+      <c r="G6" t="s">
+        <v>18</v>
+      </c>
+      <c r="H6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I6" t="s">
+        <v>20</v>
+      </c>
+      <c r="J6" t="s">
+        <v>21</v>
+      </c>
+      <c r="K6" t="s">
+        <v>44</v>
       </c>
       <c r="L6">
         <v>15</v>
       </c>
-      <c r="M6" t="str">
-        <v>21020002, 21020004, 21020088, 21020100</v>
+      <c r="M6" t="s">
+        <v>45</v>
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M6"/>
+    <ignoredError sqref="A1:M4 A6:M6 A5:H5 K5:M5" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>